<commit_message>
setting up for scrapping minutes 60 hospitals in queue
</commit_message>
<xml_diff>
--- a/roles/minutes/ResearchOnMinutes/BoardMinuteLocationFile_v2.xlsx
+++ b/roles/minutes/ResearchOnMinutes/BoardMinuteLocationFile_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HospitalIntelligenceR\roles\minutes\ResearchOnMinutes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0F1F69-7B1E-4FCC-9749-2343DD45E32A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D011846-B245-4D5C-80F5-454AF31B53B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="380" windowWidth="23980" windowHeight="15260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BoardMinutes" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1139" uniqueCount="519">
   <si>
     <t>fac</t>
   </si>
@@ -1575,6 +1575,12 @@
   </si>
   <si>
     <t>https://www.womenscollegehospital.ca/who-we-are/board-of-directors/</t>
+  </si>
+  <si>
+    <t>7:38a</t>
+  </si>
+  <si>
+    <t>4:15p</t>
   </si>
 </sst>
 </file>
@@ -6616,7 +6622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2177B12B-AAA9-470B-B19E-F75FE0A833B7}">
-  <dimension ref="A2:E7"/>
+  <dimension ref="A2:E9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.6328125" customWidth="1"/>
@@ -6715,6 +6721,40 @@
         <v>515</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="7">
+        <v>46178</v>
+      </c>
+      <c r="B8">
+        <v>118</v>
+      </c>
+      <c r="C8">
+        <v>86</v>
+      </c>
+      <c r="D8">
+        <v>73</v>
+      </c>
+      <c r="E8" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
+        <v>45814</v>
+      </c>
+      <c r="B9">
+        <v>124</v>
+      </c>
+      <c r="C9">
+        <v>87</v>
+      </c>
+      <c r="D9">
+        <v>77</v>
+      </c>
+      <c r="E9" t="s">
+        <v>517</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>